<commit_message>
feat(cms): format human-friendly CSV columns, multi-alias parser mapping, and pre-built spreadsheets
</commit_message>
<xml_diff>
--- a/Krishna_Karate_Academy_Data.xlsx
+++ b/Krishna_Karate_Academy_Data.xlsx
@@ -421,32 +421,32 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Tournament Name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Subtitle</t>
+          <t>Subtitle / Tagline</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>TargetDate</t>
+          <t>Date (YYYY-MM-DD)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>City / Venue</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Categories</t>
+          <t>Event Categories</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Status Badge</t>
         </is>
       </c>
     </row>
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>State &amp; Open Invitational Championship · 5 – 6 September</t>
+          <t>State &amp; Open Invitational Martial Arts Championship · 5 – 6 September</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -473,7 +473,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Kata Forms Division, Kumite Sparring, Cadet &amp; Senior</t>
+          <t>Kata Forms Division, Kumite Sparring, Junior &amp; Senior Cadet</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -505,7 +505,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>National Cadet Forms, Team Sparring, Senior Open</t>
+          <t>National Cadet Forms, Team Sparring Championship, Senior Open</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,7 +537,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>All 12 Belt Divisions, Kids U-18 Forms &amp; Sparring</t>
+          <t>All 12 Belt Divisions, Kids Under-18 Forms &amp; Sparring</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -557,33 +557,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Student Name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Achievement Title</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Event</t>
+          <t>Tournament Event Name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Badge</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Icon</t>
+          <t>Medal Won (Gold / Silver / Bronze)</t>
         </is>
       </c>
     </row>
@@ -608,11 +603,6 @@
           <t>INTL GOLD</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>🥇</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -635,11 +625,6 @@
           <t>INTL GOLD</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>🥇</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -662,11 +647,6 @@
           <t>NATIONAL GOLD</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>🥇</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -689,11 +669,6 @@
           <t>INTL SILVER</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>🥈</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -714,11 +689,6 @@
       <c r="D6" t="inlineStr">
         <is>
           <t>NATIONAL GOLD</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>🥇</t>
         </is>
       </c>
     </row>
@@ -739,32 +709,32 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>Black Belt Tier</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Requirement</t>
+          <t>Requirement / Experience</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>StudentName</t>
+          <t>Student Name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>StudentTitle</t>
+          <t>Role / Title</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>StudentStatus</t>
+          <t>Achievement Details</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Badge</t>
+          <t>Dan Rank</t>
         </is>
       </c>
     </row>
@@ -776,7 +746,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Chief Instructor &amp; Master Grade</t>
+          <t>Chief Instructor &amp; Master Grade · 15+ Yrs Master Experience</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -791,7 +761,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Head Examiner · 15+ Yrs Master Experience</t>
+          <t>Chennai Intl Gold Medalist · Head Examiner</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -808,7 +778,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Full 5-Year Dedicated Journey</t>
+          <t>Full 5-Year Dedicated Journey Completion &amp; Federation Accreditation</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -840,7 +810,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Full 5-Year Dedicated Journey</t>
+          <t>Full 5-Year Dedicated Journey Completion &amp; Federation Accreditation</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>